<commit_message>
feat: OCR extraction yields 122 attendees from 4 images
- Improved pytesseract/Tesseract integration with PATH configuration
- Enhanced OCR text parsing for scattered email-name patterns
- Extracted 122 attendees with emails and food restrictions
- Generated 122 encrypted QR codes ready for event
- Ready to re-run extraction with better image quality tomorrow

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/qr-generator/attendees.xlsx
+++ b/qr-generator/attendees.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F75"/>
+  <dimension ref="A1:F123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -483,7 +483,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Serge.nassar@intact.net</t>
+          <t>serge.nassar@intact.net</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -493,7 +493,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>No food for me</t>
+          <t>Count me in</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -631,7 +631,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Allergy</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -695,7 +695,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Halal</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -823,7 +823,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Gluten free</t>
+          <t>Gluten</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1015,7 +1015,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Lactose</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Pork</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1239,7 +1239,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Lactose</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1283,7 +1283,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>alexandre-Tl.morin@intact.net</t>
+          <t>alexandre-tl.morin@intact.net</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1527,7 +1527,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Carb</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1635,12 +1635,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>eric.charette@intact.net</t>
+          <t>xiao.hu@intact.net</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Eric Charette</t>
+          <t>AL .</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1667,12 +1667,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Edith.Marceau@intact.net</t>
+          <t>yanis.khati@intact.net</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Edith Marceau</t>
+          <t>AL .</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1699,12 +1699,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Charles.gascon@intact.net</t>
+          <t>beck@intact.net</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Charles Gascon</t>
+          <t>patrick</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1731,12 +1731,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Mmatthias.catherine@intact.net</t>
+          <t>faille@intact.net</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Matthias Catherine</t>
+          <t>erick</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1763,12 +1763,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>nancy.deschenes@belairdirect.com</t>
+          <t>barba@intact.net</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Nancy Deschenes</t>
+          <t>BER Maria</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1795,12 +1795,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>bienvenu.atangana@intact.net</t>
+          <t>eric.charette@intact.net</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Marc Bienvenu Atangana</t>
+          <t>Eric Charette</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1827,17 +1827,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Mario.beltran@intact.net</t>
+          <t>edith.marceau@intact.net</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Mario Beltran</t>
+          <t>Edith Marceau</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>No food for me</t>
+          <t>Count me in</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1859,12 +1859,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>dimitri.ntsoli.egolo@intact.net</t>
+          <t>charles.gascon@intact.net</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Dimitri Ntsoli Egoto</t>
+          <t>Charles Gascon</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1891,12 +1891,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>clement.thepaut@intact.net</t>
+          <t>mmatthias.catherine@intact.net</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Clement Thepaut</t>
+          <t>Matthias Catherine</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1923,12 +1923,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>alexandre.soares@intact.net</t>
+          <t>nancy.deschenes@belairdirect.com</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Alexandre Soares</t>
+          <t>Nancy Deschenes</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1955,12 +1955,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>philippe.antoniotti@intact.net</t>
+          <t>bienvenu.atangana@intact.net</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Philippe Antoniotti</t>
+          <t>Marc Bienvenu Atangana</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1987,12 +1987,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>jerre.carlos.kitio.donfack@intact.net</t>
+          <t>mario.beltran@intact.net</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Pierre Carlos Kitio Donfack</t>
+          <t>Mario Beltran</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2019,12 +2019,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>ayoub.hamidine@intact.net</t>
+          <t>dimitri.ntsoli.egolo@intact.net</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Ayoub Hamidine</t>
+          <t>Dimitri Ntsoli Egoto</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2051,12 +2051,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>alexandre.sah@intact.net</t>
+          <t>clement.thepaut@intact.net</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Alexandre Sah</t>
+          <t>Clement Thepaut</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2083,12 +2083,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>mohammed.eLamine.tali@intact.net</t>
+          <t>alexandre.soares@intact.net</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Mohammed El Amine Tali</t>
+          <t>Alexandre Soares</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2115,12 +2115,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>david-martel@intact.net</t>
+          <t>philippe.antoniotti@intact.net</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>David Martel</t>
+          <t>Philippe Antoniotti</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2147,12 +2147,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>marilyne.nguyen@intact.net</t>
+          <t>jerre.carlos.kitio.donfack@intact.net</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Marilyne Nguyen</t>
+          <t>Pierre Carlos Kitio Donfack</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2179,12 +2179,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>ryan.yi.cheng.shen@intact.net</t>
+          <t>ayoub.hamidine@intact.net</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Ryan Yi Cheng Shen</t>
+          <t>Ayoub Hamidine</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2211,12 +2211,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>lilya.benladjreb@intact.net</t>
+          <t>alexandre.sah@intact.net</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Lilya Benladjreb</t>
+          <t>Alexandre Sah</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2243,12 +2243,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>fouetieu.kom@intact.net</t>
+          <t>mohammed.elamine.tali@intact.net</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Andre-Ange Fouetieu Kom</t>
+          <t>Mohammed El Amine Tali</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2263,7 +2263,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Lactose</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2275,12 +2275,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>daneau@intact.net</t>
+          <t>david-martel@intact.net</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Satya Daneau</t>
+          <t>David Martel</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2307,12 +2307,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>franquet@intact.net</t>
+          <t>marilyne.nguyen@intact.net</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Dorothee Franquet</t>
+          <t>Marilyne Nguyen</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2339,12 +2339,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>domingues@intact.net</t>
+          <t>ryan.yi.cheng.shen@intact.net</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Patrick Domingues</t>
+          <t>Ryan Yi Cheng Shen</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2371,12 +2371,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>nadia_penagos@intact.net</t>
+          <t>lilya.benladjreb@intact.net</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Nadia Penagos</t>
+          <t>Lilya Benladjreb</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2391,7 +2391,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Gluten free</t>
+          <t>None</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -2403,12 +2403,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>dickson.chea@intact.net</t>
+          <t>fouetieu.kom@intact.net</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Dickson Chea</t>
+          <t>Andre-Ange Fouetieu Kom</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2435,12 +2435,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>danny-farkouh@intact.net</t>
+          <t>daneau@intact.net</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Danny Farkouh</t>
+          <t>Satya Daneau</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -2467,12 +2467,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>MicheLDugal@intact.net</t>
+          <t>franquet@intact.net</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Michel Dugal</t>
+          <t>Dorothee Franquet</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2499,12 +2499,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>etienne.carle@intact.net</t>
+          <t>domingues@intact.net</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Etienne Carle</t>
+          <t>Patrick Domingues</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2531,12 +2531,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>burton@intact.net</t>
+          <t>nadia_penagos@intact.net</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>George Burton</t>
+          <t>Nadia Penagos</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2551,7 +2551,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Vegetarian</t>
+          <t>Gluten</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -2563,17 +2563,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>merouane.bouloudene@intact.net</t>
+          <t>dickson.chea@intact.net</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Merouane Bouloudene</t>
+          <t>Dickson Chea</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>No food for me</t>
+          <t>Count me in</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2595,12 +2595,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>yacine.dahak@intact.net</t>
+          <t>danny-farkouh@intact.net</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Yacine Dahak</t>
+          <t>Danny Farkouh</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -2627,12 +2627,12 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>olatayo.elegbede@intact.net</t>
+          <t>micheldugal@intact.net</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Olatayo Elegbede</t>
+          <t>Michel Dugal</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -2659,12 +2659,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>moustavi-al-manee.haque@intact.net</t>
+          <t>etienne.carle@intact.net</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Moustavi-Al-Manee Haque</t>
+          <t>Etienne Carle</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -2679,7 +2679,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Carb</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -2691,12 +2691,12 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>bibeau@intact.net</t>
+          <t>burton@intact.net</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Joanie Bibeau</t>
+          <t>George Burton</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -2711,7 +2711,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Vegetarian</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -2723,12 +2723,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>marc.laberge@intact.net</t>
+          <t>merouane.bouloudene@intact.net</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Marc Laberge</t>
+          <t>Merouane Bouloudene</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -2755,12 +2755,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>fiamma.saragosa@intact.net</t>
+          <t>yacine.dahak@intact.net</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Fiamma Saragosa</t>
+          <t>Yacine Dahak</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -2775,7 +2775,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Halal</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -2787,30 +2787,1566 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>karLxavier.dagenais@intact.net</t>
+          <t>olatayo.elegbede@intact.net</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
+          <t>Olatayo Elegbede</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>moustavi-al-manee.haque@intact.net</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Moustavi-Al-Manee Haque</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Pork</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>bibeau@intact.net</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Joanie Bibeau</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>marc.laberge@intact.net</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Marc Laberge</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>fiamma.saragosa@intact.net</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Fiamma Saragosa</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>karlxavier.dagenais@intact.net</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
           <t>Karl Xavier Dagenais</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>Count me in</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>Count me in</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="F75" t="inlineStr">
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>lon@intact.net</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>geal</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>raoui@intact.net</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>geal</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>florent.te.bail@intact.net</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>FUP)</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>mathis.belanger@intact.net</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>s()-</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>tringa@intact.net</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>BU axel</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>hossein.hajisoleimani@intact.net</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Bly</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>paquet@intact.net</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>julie-.</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>cedric.pharand@intact.net</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>gl)</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>imen.mhamdi@intact.net</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>BEL)</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>brian-blosser@intact.net</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>BebY</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>rivard@intact.net</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>BEK) marie.eve</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>geran@intact.net</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>gbC) mickeel</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>hari-mr@intact.net</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>pel</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>zammit@intact.net</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>pee paul</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>jean-sebastien_tasse@intact.net</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>BBL</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>gamien-antoine@intact.net</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>get)</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>duchemin@intact.net</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>p-) pierre.</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>valois@intact.net</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>gr) marcos</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>simen@intact.net</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>yannick jordan. monthe</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>hamit.pena.sierra@intact.net</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Be)</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>john.paragas@intact.net</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>alexia.teissier@intact.net</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>eC)</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>louis-philippe.cregheur@intact.net</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Btt)</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>anneli.west@intact.net</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>BUS</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>chloe.bosch@intact.net</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>houda.bagane@intact.net</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>BUX</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>afsaneh.khan@belairdirect.com</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>BLY</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>mathew-kanner@intact.net</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>pt)</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>vishruti.gopani@intact.net</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>BtS</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>oumaima.charifa.el.khayiri@intact.net</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>b(t)</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>lotfi-meklati@intact.net</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>BLS</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>gavoud.ramezani.kermani@intact.net</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>p(y</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>chantale.laberge@intact.net</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>BUX</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>brisson@intact.net</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>BUS camille</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>alae.hassoun@intact.net</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>pl)</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>latendresse@belairdirect.com</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>pts) karine</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>alexander.alessi@intact.net</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Bt)</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>nestine.moulay-abdallah@intact.net</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>BtS-)</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>dilleltahmani@intact.net</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Bet)</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>tebbji@intact.net</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>pu yassine</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>mayvin.tamasawmy@intact.net</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>BEG)</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>vincent-bernier@intact.net</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>BUg</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>Squad 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>st-pierre@intact.net</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>ELEN marc</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Count me in</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
         <is>
           <t>Squad 1</t>
         </is>

</xml_diff>